<commit_message>
Update readme, update template, add Excel download to bottom of page and hide data source at start
</commit_message>
<xml_diff>
--- a/public/excel template/Template.xlsx
+++ b/public/excel template/Template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADADAFDD-440A-42BD-93B4-A2237623D618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0356DF3C-3447-4229-A2F9-B79D8D7C8AF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BECE5613-4CE6-4BB7-8FF1-F4E60925457F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{BECE5613-4CE6-4BB7-8FF1-F4E60925457F}"/>
   </bookViews>
   <sheets>
     <sheet name="Small" sheetId="2" r:id="rId1"/>
@@ -572,12 +572,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
-    <dxf>
-      <fill>
-        <patternFill patternType="gray125"/>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="lightGray"/>
@@ -586,98 +581,6 @@
     <dxf>
       <fill>
         <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="lightGray"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
       </fill>
     </dxf>
   </dxfs>
@@ -1014,9 +917,9 @@
   <dimension ref="A1:Z18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" customWidth="1"/>
+    <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="9" width="15.140625" customWidth="1"/>
-    <col min="10" max="11" width="4.7109375" style="5" customWidth="1"/>
+    <col min="10" max="11" width="5.28515625" style="5" customWidth="1"/>
     <col min="12" max="12" width="2.42578125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1099,11 +1002,11 @@
       <c r="H5" s="10"/>
       <c r="I5" s="10"/>
       <c r="J5" s="38">
-        <v>45825</v>
+        <v>45916</v>
       </c>
       <c r="K5" s="38">
         <f>J5+6</f>
-        <v>45831</v>
+        <v>45922</v>
       </c>
       <c r="M5" s="13"/>
       <c r="N5" s="13"/>
@@ -1132,11 +1035,11 @@
       <c r="I6" s="15"/>
       <c r="J6" s="35">
         <f>J5+7</f>
-        <v>45832</v>
+        <v>45923</v>
       </c>
       <c r="K6" s="35">
         <f>K5+7</f>
-        <v>45838</v>
+        <v>45929</v>
       </c>
       <c r="M6" s="13"/>
       <c r="N6" s="16"/>
@@ -1166,11 +1069,11 @@
       <c r="I7" s="10"/>
       <c r="J7" s="35">
         <f t="shared" ref="J7:K16" si="0">J6+7</f>
-        <v>45839</v>
+        <v>45930</v>
       </c>
       <c r="K7" s="35">
         <f t="shared" si="0"/>
-        <v>45845</v>
+        <v>45936</v>
       </c>
       <c r="M7" s="13"/>
       <c r="N7" s="17"/>
@@ -1201,11 +1104,11 @@
       <c r="I8" s="10"/>
       <c r="J8" s="35">
         <f t="shared" si="0"/>
-        <v>45846</v>
+        <v>45937</v>
       </c>
       <c r="K8" s="35">
         <f t="shared" si="0"/>
-        <v>45852</v>
+        <v>45943</v>
       </c>
       <c r="M8" s="13"/>
       <c r="N8" s="19"/>
@@ -1229,11 +1132,11 @@
       <c r="I9" s="10"/>
       <c r="J9" s="35">
         <f t="shared" si="0"/>
-        <v>45853</v>
+        <v>45944</v>
       </c>
       <c r="K9" s="35">
         <f t="shared" si="0"/>
-        <v>45859</v>
+        <v>45950</v>
       </c>
       <c r="M9" s="13"/>
       <c r="N9" s="17"/>
@@ -1257,11 +1160,11 @@
       <c r="I10" s="10"/>
       <c r="J10" s="35">
         <f t="shared" si="0"/>
-        <v>45860</v>
+        <v>45951</v>
       </c>
       <c r="K10" s="35">
         <f t="shared" si="0"/>
-        <v>45866</v>
+        <v>45957</v>
       </c>
       <c r="M10" s="13"/>
       <c r="N10" s="17"/>
@@ -1285,11 +1188,11 @@
       <c r="I11" s="10"/>
       <c r="J11" s="35">
         <f t="shared" si="0"/>
-        <v>45867</v>
+        <v>45958</v>
       </c>
       <c r="K11" s="35">
         <f t="shared" si="0"/>
-        <v>45873</v>
+        <v>45964</v>
       </c>
       <c r="M11" s="13"/>
       <c r="N11" s="17"/>
@@ -1313,11 +1216,11 @@
       <c r="I12" s="10"/>
       <c r="J12" s="35">
         <f t="shared" si="0"/>
-        <v>45874</v>
+        <v>45965</v>
       </c>
       <c r="K12" s="35">
         <f t="shared" si="0"/>
-        <v>45880</v>
+        <v>45971</v>
       </c>
       <c r="M12" s="13"/>
       <c r="N12" s="17"/>
@@ -1341,11 +1244,11 @@
       <c r="I13" s="10"/>
       <c r="J13" s="35">
         <f t="shared" si="0"/>
-        <v>45881</v>
+        <v>45972</v>
       </c>
       <c r="K13" s="35">
         <f t="shared" si="0"/>
-        <v>45887</v>
+        <v>45978</v>
       </c>
       <c r="M13" s="13"/>
       <c r="N13" s="17"/>
@@ -1369,11 +1272,11 @@
       <c r="I14" s="10"/>
       <c r="J14" s="35">
         <f t="shared" si="0"/>
-        <v>45888</v>
+        <v>45979</v>
       </c>
       <c r="K14" s="35">
         <f t="shared" si="0"/>
-        <v>45894</v>
+        <v>45985</v>
       </c>
       <c r="M14" s="13"/>
       <c r="N14" s="17"/>
@@ -1397,11 +1300,11 @@
       <c r="I15" s="10"/>
       <c r="J15" s="35">
         <f t="shared" si="0"/>
-        <v>45895</v>
+        <v>45986</v>
       </c>
       <c r="K15" s="35">
         <f t="shared" si="0"/>
-        <v>45901</v>
+        <v>45992</v>
       </c>
       <c r="M15" s="13"/>
       <c r="N15" s="17"/>
@@ -1425,11 +1328,11 @@
       <c r="I16" s="22"/>
       <c r="J16" s="52">
         <f t="shared" si="0"/>
-        <v>45902</v>
+        <v>45993</v>
       </c>
       <c r="K16" s="52">
         <f t="shared" si="0"/>
-        <v>45908</v>
+        <v>45999</v>
       </c>
       <c r="M16" s="13"/>
       <c r="N16" s="17"/>
@@ -1462,7 +1365,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="B5:I16">
-    <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="%">
+    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="%">
       <formula>NOT(ISERROR(SEARCH("%",B5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -1475,16 +1378,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D7E8E88F-E57D-4595-BFF0-FC906AD171D4}">
   <sheetPr codeName="Sheet11"/>
-  <dimension ref="A1:EV18"/>
+  <dimension ref="A1:FK18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" customWidth="1"/>
-    <col min="2" max="135" width="14.7109375" customWidth="1"/>
-    <col min="136" max="137" width="5.42578125" style="5" customWidth="1"/>
-    <col min="138" max="138" width="2.42578125" customWidth="1"/>
+    <col min="2" max="150" width="14.7109375" customWidth="1"/>
+    <col min="151" max="152" width="5.42578125" style="5" customWidth="1"/>
+    <col min="153" max="153" width="2.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:152" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:167" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1622,8 +1525,23 @@
       <c r="EC1" s="49"/>
       <c r="ED1" s="49"/>
       <c r="EE1" s="49"/>
+      <c r="EF1" s="49"/>
+      <c r="EG1" s="49"/>
+      <c r="EH1" s="49"/>
+      <c r="EI1" s="49"/>
+      <c r="EJ1" s="49"/>
+      <c r="EK1" s="49"/>
+      <c r="EL1" s="49"/>
+      <c r="EM1" s="49"/>
+      <c r="EN1" s="49"/>
+      <c r="EO1" s="49"/>
+      <c r="EP1" s="49"/>
+      <c r="EQ1" s="49"/>
+      <c r="ER1" s="49"/>
+      <c r="ES1" s="49"/>
+      <c r="ET1" s="49"/>
     </row>
-    <row r="2" spans="1:152" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:167" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -1761,8 +1679,23 @@
       <c r="EC2" s="4"/>
       <c r="ED2" s="4"/>
       <c r="EE2" s="4"/>
+      <c r="EF2" s="4"/>
+      <c r="EG2" s="4"/>
+      <c r="EH2" s="4"/>
+      <c r="EI2" s="4"/>
+      <c r="EJ2" s="4"/>
+      <c r="EK2" s="4"/>
+      <c r="EL2" s="4"/>
+      <c r="EM2" s="4"/>
+      <c r="EN2" s="4"/>
+      <c r="EO2" s="4"/>
+      <c r="EP2" s="4"/>
+      <c r="EQ2" s="4"/>
+      <c r="ER2" s="4"/>
+      <c r="ES2" s="4"/>
+      <c r="ET2" s="4"/>
     </row>
-    <row r="3" spans="1:152" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:167" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1900,8 +1833,23 @@
       <c r="EC3" s="4"/>
       <c r="ED3" s="4"/>
       <c r="EE3" s="4"/>
+      <c r="EF3" s="4"/>
+      <c r="EG3" s="4"/>
+      <c r="EH3" s="4"/>
+      <c r="EI3" s="4"/>
+      <c r="EJ3" s="4"/>
+      <c r="EK3" s="4"/>
+      <c r="EL3" s="4"/>
+      <c r="EM3" s="4"/>
+      <c r="EN3" s="4"/>
+      <c r="EO3" s="4"/>
+      <c r="EP3" s="4"/>
+      <c r="EQ3" s="4"/>
+      <c r="ER3" s="4"/>
+      <c r="ES3" s="4"/>
+      <c r="ET3" s="4"/>
     </row>
-    <row r="4" spans="1:152" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:167" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
@@ -2039,14 +1987,29 @@
       <c r="EC4" s="50"/>
       <c r="ED4" s="50"/>
       <c r="EE4" s="50"/>
-      <c r="EF4" s="7" t="s">
+      <c r="EF4" s="50"/>
+      <c r="EG4" s="50"/>
+      <c r="EH4" s="50"/>
+      <c r="EI4" s="50"/>
+      <c r="EJ4" s="50"/>
+      <c r="EK4" s="50"/>
+      <c r="EL4" s="50"/>
+      <c r="EM4" s="50"/>
+      <c r="EN4" s="50"/>
+      <c r="EO4" s="50"/>
+      <c r="EP4" s="50"/>
+      <c r="EQ4" s="50"/>
+      <c r="ER4" s="50"/>
+      <c r="ES4" s="50"/>
+      <c r="ET4" s="50"/>
+      <c r="EU4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="EG4" s="7" t="s">
+      <c r="EV4" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:152" ht="39" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:167" ht="39" customHeight="1" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="8">
         <v>1</v>
       </c>
@@ -2184,27 +2147,42 @@
       <c r="EC5" s="10"/>
       <c r="ED5" s="10"/>
       <c r="EE5" s="10"/>
-      <c r="EF5" s="11">
-        <v>45825</v>
-      </c>
-      <c r="EG5" s="12">
-        <f>EF5+6</f>
-        <v>45831</v>
-      </c>
-      <c r="EI5" s="13"/>
-      <c r="EJ5" s="13"/>
-      <c r="EK5" s="13"/>
-      <c r="EL5" s="13"/>
-      <c r="EM5" s="13"/>
-      <c r="EN5" s="13"/>
-      <c r="EO5" s="13"/>
-      <c r="EP5" s="13"/>
-      <c r="EQ5" s="13"/>
-      <c r="ER5" s="13"/>
-      <c r="ES5" s="13"/>
-      <c r="ET5" s="13"/>
+      <c r="EF5" s="10"/>
+      <c r="EG5" s="10"/>
+      <c r="EH5" s="10"/>
+      <c r="EI5" s="10"/>
+      <c r="EJ5" s="10"/>
+      <c r="EK5" s="10"/>
+      <c r="EL5" s="10"/>
+      <c r="EM5" s="10"/>
+      <c r="EN5" s="10"/>
+      <c r="EO5" s="10"/>
+      <c r="EP5" s="10"/>
+      <c r="EQ5" s="10"/>
+      <c r="ER5" s="10"/>
+      <c r="ES5" s="10"/>
+      <c r="ET5" s="10"/>
+      <c r="EU5" s="11">
+        <v>45916</v>
+      </c>
+      <c r="EV5" s="12">
+        <f>EU5+6</f>
+        <v>45922</v>
+      </c>
+      <c r="EX5" s="13"/>
+      <c r="EY5" s="13"/>
+      <c r="EZ5" s="13"/>
+      <c r="FA5" s="13"/>
+      <c r="FB5" s="13"/>
+      <c r="FC5" s="13"/>
+      <c r="FD5" s="13"/>
+      <c r="FE5" s="13"/>
+      <c r="FF5" s="13"/>
+      <c r="FG5" s="13"/>
+      <c r="FH5" s="13"/>
+      <c r="FI5" s="13"/>
     </row>
-    <row r="6" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="14">
         <v>2</v>
       </c>
@@ -2341,30 +2319,45 @@
       <c r="EB6" s="15"/>
       <c r="EC6" s="15"/>
       <c r="ED6" s="15"/>
-      <c r="EE6" s="10"/>
-      <c r="EF6" s="11">
-        <f>EF5+7</f>
-        <v>45832</v>
-      </c>
-      <c r="EG6" s="12">
-        <f>EG5+7</f>
-        <v>45838</v>
-      </c>
-      <c r="EI6" s="13"/>
-      <c r="EJ6" s="16"/>
-      <c r="EK6" s="16"/>
-      <c r="EL6" s="16"/>
-      <c r="EM6" s="16"/>
-      <c r="EN6" s="16"/>
-      <c r="EO6" s="17"/>
-      <c r="EP6" s="13"/>
-      <c r="EQ6" s="13"/>
-      <c r="ER6" s="13"/>
-      <c r="ES6" s="13"/>
-      <c r="ET6" s="13"/>
-      <c r="EU6" s="13"/>
+      <c r="EE6" s="15"/>
+      <c r="EF6" s="15"/>
+      <c r="EG6" s="15"/>
+      <c r="EH6" s="15"/>
+      <c r="EI6" s="15"/>
+      <c r="EJ6" s="15"/>
+      <c r="EK6" s="15"/>
+      <c r="EL6" s="15"/>
+      <c r="EM6" s="15"/>
+      <c r="EN6" s="15"/>
+      <c r="EO6" s="15"/>
+      <c r="EP6" s="15"/>
+      <c r="EQ6" s="15"/>
+      <c r="ER6" s="15"/>
+      <c r="ES6" s="15"/>
+      <c r="ET6" s="10"/>
+      <c r="EU6" s="11">
+        <f>EU5+7</f>
+        <v>45923</v>
+      </c>
+      <c r="EV6" s="12">
+        <f>EV5+7</f>
+        <v>45929</v>
+      </c>
+      <c r="EX6" s="13"/>
+      <c r="EY6" s="16"/>
+      <c r="EZ6" s="16"/>
+      <c r="FA6" s="16"/>
+      <c r="FB6" s="16"/>
+      <c r="FC6" s="16"/>
+      <c r="FD6" s="17"/>
+      <c r="FE6" s="13"/>
+      <c r="FF6" s="13"/>
+      <c r="FG6" s="13"/>
+      <c r="FH6" s="13"/>
+      <c r="FI6" s="13"/>
+      <c r="FJ6" s="13"/>
     </row>
-    <row r="7" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="14">
         <v>3</v>
       </c>
@@ -2500,32 +2493,47 @@
       <c r="EA7" s="10"/>
       <c r="EB7" s="10"/>
       <c r="EC7" s="10"/>
-      <c r="ED7" s="25"/>
+      <c r="ED7" s="10"/>
       <c r="EE7" s="10"/>
-      <c r="EF7" s="11">
-        <f t="shared" ref="EF7:EG16" si="0">EF6+7</f>
-        <v>45839</v>
-      </c>
-      <c r="EG7" s="12">
+      <c r="EF7" s="10"/>
+      <c r="EG7" s="10"/>
+      <c r="EH7" s="10"/>
+      <c r="EI7" s="10"/>
+      <c r="EJ7" s="10"/>
+      <c r="EK7" s="10"/>
+      <c r="EL7" s="10"/>
+      <c r="EM7" s="10"/>
+      <c r="EN7" s="10"/>
+      <c r="EO7" s="10"/>
+      <c r="EP7" s="10"/>
+      <c r="EQ7" s="10"/>
+      <c r="ER7" s="10"/>
+      <c r="ES7" s="25"/>
+      <c r="ET7" s="10"/>
+      <c r="EU7" s="11">
+        <f t="shared" ref="EU7:EV16" si="0">EU6+7</f>
+        <v>45930</v>
+      </c>
+      <c r="EV7" s="12">
         <f t="shared" si="0"/>
-        <v>45845</v>
-      </c>
-      <c r="EI7" s="13"/>
-      <c r="EJ7" s="17"/>
-      <c r="EK7" s="17"/>
-      <c r="EL7" s="18"/>
-      <c r="EM7" s="18"/>
-      <c r="EN7" s="17"/>
-      <c r="EO7" s="19"/>
-      <c r="EP7" s="13"/>
-      <c r="EQ7" s="13"/>
-      <c r="ER7" s="13"/>
-      <c r="ES7" s="13"/>
-      <c r="ET7" s="13"/>
-      <c r="EU7" s="13"/>
-      <c r="EV7" s="13"/>
+        <v>45936</v>
+      </c>
+      <c r="EX7" s="13"/>
+      <c r="EY7" s="17"/>
+      <c r="EZ7" s="17"/>
+      <c r="FA7" s="18"/>
+      <c r="FB7" s="18"/>
+      <c r="FC7" s="17"/>
+      <c r="FD7" s="19"/>
+      <c r="FE7" s="13"/>
+      <c r="FF7" s="13"/>
+      <c r="FG7" s="13"/>
+      <c r="FH7" s="13"/>
+      <c r="FI7" s="13"/>
+      <c r="FJ7" s="13"/>
+      <c r="FK7" s="13"/>
     </row>
-    <row r="8" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="14">
         <v>4</v>
       </c>
@@ -2663,23 +2671,38 @@
       <c r="EC8" s="10"/>
       <c r="ED8" s="10"/>
       <c r="EE8" s="10"/>
-      <c r="EF8" s="11">
+      <c r="EF8" s="10"/>
+      <c r="EG8" s="10"/>
+      <c r="EH8" s="10"/>
+      <c r="EI8" s="10"/>
+      <c r="EJ8" s="10"/>
+      <c r="EK8" s="10"/>
+      <c r="EL8" s="10"/>
+      <c r="EM8" s="10"/>
+      <c r="EN8" s="10"/>
+      <c r="EO8" s="10"/>
+      <c r="EP8" s="10"/>
+      <c r="EQ8" s="10"/>
+      <c r="ER8" s="10"/>
+      <c r="ES8" s="10"/>
+      <c r="ET8" s="10"/>
+      <c r="EU8" s="11">
         <f t="shared" si="0"/>
-        <v>45846</v>
-      </c>
-      <c r="EG8" s="12">
+        <v>45937</v>
+      </c>
+      <c r="EV8" s="12">
         <f t="shared" si="0"/>
-        <v>45852</v>
-      </c>
-      <c r="EI8" s="13"/>
-      <c r="EJ8" s="19"/>
-      <c r="EK8" s="19"/>
-      <c r="EL8" s="20"/>
-      <c r="EM8" s="20"/>
-      <c r="EN8" s="19"/>
-      <c r="EO8" s="17"/>
+        <v>45943</v>
+      </c>
+      <c r="EX8" s="13"/>
+      <c r="EY8" s="19"/>
+      <c r="EZ8" s="19"/>
+      <c r="FA8" s="20"/>
+      <c r="FB8" s="20"/>
+      <c r="FC8" s="19"/>
+      <c r="FD8" s="17"/>
     </row>
-    <row r="9" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="14">
         <v>5</v>
       </c>
@@ -2817,23 +2840,38 @@
       <c r="EC9" s="10"/>
       <c r="ED9" s="10"/>
       <c r="EE9" s="10"/>
-      <c r="EF9" s="11">
+      <c r="EF9" s="10"/>
+      <c r="EG9" s="10"/>
+      <c r="EH9" s="10"/>
+      <c r="EI9" s="10"/>
+      <c r="EJ9" s="10"/>
+      <c r="EK9" s="10"/>
+      <c r="EL9" s="10"/>
+      <c r="EM9" s="10"/>
+      <c r="EN9" s="10"/>
+      <c r="EO9" s="10"/>
+      <c r="EP9" s="10"/>
+      <c r="EQ9" s="10"/>
+      <c r="ER9" s="10"/>
+      <c r="ES9" s="10"/>
+      <c r="ET9" s="10"/>
+      <c r="EU9" s="11">
         <f t="shared" si="0"/>
-        <v>45853</v>
-      </c>
-      <c r="EG9" s="12">
+        <v>45944</v>
+      </c>
+      <c r="EV9" s="12">
         <f t="shared" si="0"/>
-        <v>45859</v>
-      </c>
-      <c r="EI9" s="13"/>
-      <c r="EJ9" s="17"/>
-      <c r="EK9" s="17"/>
-      <c r="EL9" s="18"/>
-      <c r="EM9" s="18"/>
-      <c r="EN9" s="17"/>
-      <c r="EO9" s="17"/>
+        <v>45950</v>
+      </c>
+      <c r="EX9" s="13"/>
+      <c r="EY9" s="17"/>
+      <c r="EZ9" s="17"/>
+      <c r="FA9" s="18"/>
+      <c r="FB9" s="18"/>
+      <c r="FC9" s="17"/>
+      <c r="FD9" s="17"/>
     </row>
-    <row r="10" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="14">
         <v>6</v>
       </c>
@@ -2971,23 +3009,38 @@
       <c r="EC10" s="10"/>
       <c r="ED10" s="10"/>
       <c r="EE10" s="10"/>
-      <c r="EF10" s="11">
+      <c r="EF10" s="10"/>
+      <c r="EG10" s="10"/>
+      <c r="EH10" s="10"/>
+      <c r="EI10" s="10"/>
+      <c r="EJ10" s="10"/>
+      <c r="EK10" s="10"/>
+      <c r="EL10" s="10"/>
+      <c r="EM10" s="10"/>
+      <c r="EN10" s="10"/>
+      <c r="EO10" s="10"/>
+      <c r="EP10" s="10"/>
+      <c r="EQ10" s="10"/>
+      <c r="ER10" s="10"/>
+      <c r="ES10" s="10"/>
+      <c r="ET10" s="10"/>
+      <c r="EU10" s="11">
         <f t="shared" si="0"/>
-        <v>45860</v>
-      </c>
-      <c r="EG10" s="12">
+        <v>45951</v>
+      </c>
+      <c r="EV10" s="12">
         <f t="shared" si="0"/>
-        <v>45866</v>
-      </c>
-      <c r="EI10" s="13"/>
-      <c r="EJ10" s="17"/>
-      <c r="EK10" s="17"/>
-      <c r="EL10" s="18"/>
-      <c r="EM10" s="18"/>
-      <c r="EN10" s="17"/>
-      <c r="EO10" s="17"/>
+        <v>45957</v>
+      </c>
+      <c r="EX10" s="13"/>
+      <c r="EY10" s="17"/>
+      <c r="EZ10" s="17"/>
+      <c r="FA10" s="18"/>
+      <c r="FB10" s="18"/>
+      <c r="FC10" s="17"/>
+      <c r="FD10" s="17"/>
     </row>
-    <row r="11" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14">
         <v>7</v>
       </c>
@@ -3125,23 +3178,38 @@
       <c r="EC11" s="10"/>
       <c r="ED11" s="10"/>
       <c r="EE11" s="10"/>
-      <c r="EF11" s="11">
+      <c r="EF11" s="10"/>
+      <c r="EG11" s="10"/>
+      <c r="EH11" s="10"/>
+      <c r="EI11" s="10"/>
+      <c r="EJ11" s="10"/>
+      <c r="EK11" s="10"/>
+      <c r="EL11" s="10"/>
+      <c r="EM11" s="10"/>
+      <c r="EN11" s="10"/>
+      <c r="EO11" s="10"/>
+      <c r="EP11" s="10"/>
+      <c r="EQ11" s="10"/>
+      <c r="ER11" s="10"/>
+      <c r="ES11" s="10"/>
+      <c r="ET11" s="10"/>
+      <c r="EU11" s="11">
         <f t="shared" si="0"/>
-        <v>45867</v>
-      </c>
-      <c r="EG11" s="12">
+        <v>45958</v>
+      </c>
+      <c r="EV11" s="12">
         <f t="shared" si="0"/>
-        <v>45873</v>
-      </c>
-      <c r="EI11" s="13"/>
-      <c r="EJ11" s="17"/>
-      <c r="EK11" s="17"/>
-      <c r="EL11" s="18"/>
-      <c r="EM11" s="18"/>
-      <c r="EN11" s="17"/>
-      <c r="EO11" s="17"/>
+        <v>45964</v>
+      </c>
+      <c r="EX11" s="13"/>
+      <c r="EY11" s="17"/>
+      <c r="EZ11" s="17"/>
+      <c r="FA11" s="18"/>
+      <c r="FB11" s="18"/>
+      <c r="FC11" s="17"/>
+      <c r="FD11" s="17"/>
     </row>
-    <row r="12" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="14">
         <v>8</v>
       </c>
@@ -3279,23 +3347,38 @@
       <c r="EC12" s="10"/>
       <c r="ED12" s="10"/>
       <c r="EE12" s="10"/>
-      <c r="EF12" s="11">
+      <c r="EF12" s="10"/>
+      <c r="EG12" s="10"/>
+      <c r="EH12" s="10"/>
+      <c r="EI12" s="10"/>
+      <c r="EJ12" s="10"/>
+      <c r="EK12" s="10"/>
+      <c r="EL12" s="10"/>
+      <c r="EM12" s="10"/>
+      <c r="EN12" s="10"/>
+      <c r="EO12" s="10"/>
+      <c r="EP12" s="10"/>
+      <c r="EQ12" s="10"/>
+      <c r="ER12" s="10"/>
+      <c r="ES12" s="10"/>
+      <c r="ET12" s="10"/>
+      <c r="EU12" s="11">
         <f t="shared" si="0"/>
-        <v>45874</v>
-      </c>
-      <c r="EG12" s="12">
+        <v>45965</v>
+      </c>
+      <c r="EV12" s="12">
         <f t="shared" si="0"/>
-        <v>45880</v>
-      </c>
-      <c r="EI12" s="13"/>
-      <c r="EJ12" s="17"/>
-      <c r="EK12" s="17"/>
-      <c r="EL12" s="18"/>
-      <c r="EM12" s="18"/>
-      <c r="EN12" s="17"/>
-      <c r="EO12" s="17"/>
+        <v>45971</v>
+      </c>
+      <c r="EX12" s="13"/>
+      <c r="EY12" s="17"/>
+      <c r="EZ12" s="17"/>
+      <c r="FA12" s="18"/>
+      <c r="FB12" s="18"/>
+      <c r="FC12" s="17"/>
+      <c r="FD12" s="17"/>
     </row>
-    <row r="13" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="14">
         <v>9</v>
       </c>
@@ -3433,23 +3516,38 @@
       <c r="EC13" s="10"/>
       <c r="ED13" s="10"/>
       <c r="EE13" s="10"/>
-      <c r="EF13" s="11">
+      <c r="EF13" s="10"/>
+      <c r="EG13" s="10"/>
+      <c r="EH13" s="10"/>
+      <c r="EI13" s="10"/>
+      <c r="EJ13" s="10"/>
+      <c r="EK13" s="10"/>
+      <c r="EL13" s="10"/>
+      <c r="EM13" s="10"/>
+      <c r="EN13" s="10"/>
+      <c r="EO13" s="10"/>
+      <c r="EP13" s="10"/>
+      <c r="EQ13" s="10"/>
+      <c r="ER13" s="10"/>
+      <c r="ES13" s="10"/>
+      <c r="ET13" s="10"/>
+      <c r="EU13" s="11">
         <f t="shared" si="0"/>
-        <v>45881</v>
-      </c>
-      <c r="EG13" s="12">
+        <v>45972</v>
+      </c>
+      <c r="EV13" s="12">
         <f t="shared" si="0"/>
-        <v>45887</v>
-      </c>
-      <c r="EI13" s="13"/>
-      <c r="EJ13" s="17"/>
-      <c r="EK13" s="17"/>
-      <c r="EL13" s="18"/>
-      <c r="EM13" s="18"/>
-      <c r="EN13" s="17"/>
-      <c r="EO13" s="17"/>
+        <v>45978</v>
+      </c>
+      <c r="EX13" s="13"/>
+      <c r="EY13" s="17"/>
+      <c r="EZ13" s="17"/>
+      <c r="FA13" s="18"/>
+      <c r="FB13" s="18"/>
+      <c r="FC13" s="17"/>
+      <c r="FD13" s="17"/>
     </row>
-    <row r="14" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14">
         <v>10</v>
       </c>
@@ -3587,23 +3685,38 @@
       <c r="EC14" s="10"/>
       <c r="ED14" s="10"/>
       <c r="EE14" s="10"/>
-      <c r="EF14" s="11">
+      <c r="EF14" s="10"/>
+      <c r="EG14" s="10"/>
+      <c r="EH14" s="10"/>
+      <c r="EI14" s="10"/>
+      <c r="EJ14" s="10"/>
+      <c r="EK14" s="10"/>
+      <c r="EL14" s="10"/>
+      <c r="EM14" s="10"/>
+      <c r="EN14" s="10"/>
+      <c r="EO14" s="10"/>
+      <c r="EP14" s="10"/>
+      <c r="EQ14" s="10"/>
+      <c r="ER14" s="10"/>
+      <c r="ES14" s="10"/>
+      <c r="ET14" s="10"/>
+      <c r="EU14" s="11">
         <f t="shared" si="0"/>
-        <v>45888</v>
-      </c>
-      <c r="EG14" s="12">
+        <v>45979</v>
+      </c>
+      <c r="EV14" s="12">
         <f t="shared" si="0"/>
-        <v>45894</v>
-      </c>
-      <c r="EI14" s="13"/>
-      <c r="EJ14" s="17"/>
-      <c r="EK14" s="17"/>
-      <c r="EL14" s="18"/>
-      <c r="EM14" s="18"/>
-      <c r="EN14" s="17"/>
-      <c r="EO14" s="17"/>
+        <v>45985</v>
+      </c>
+      <c r="EX14" s="13"/>
+      <c r="EY14" s="17"/>
+      <c r="EZ14" s="17"/>
+      <c r="FA14" s="18"/>
+      <c r="FB14" s="18"/>
+      <c r="FC14" s="17"/>
+      <c r="FD14" s="17"/>
     </row>
-    <row r="15" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="14">
         <v>11</v>
       </c>
@@ -3741,23 +3854,38 @@
       <c r="EC15" s="10"/>
       <c r="ED15" s="10"/>
       <c r="EE15" s="10"/>
-      <c r="EF15" s="11">
+      <c r="EF15" s="10"/>
+      <c r="EG15" s="10"/>
+      <c r="EH15" s="10"/>
+      <c r="EI15" s="10"/>
+      <c r="EJ15" s="10"/>
+      <c r="EK15" s="10"/>
+      <c r="EL15" s="10"/>
+      <c r="EM15" s="10"/>
+      <c r="EN15" s="10"/>
+      <c r="EO15" s="10"/>
+      <c r="EP15" s="10"/>
+      <c r="EQ15" s="10"/>
+      <c r="ER15" s="10"/>
+      <c r="ES15" s="10"/>
+      <c r="ET15" s="10"/>
+      <c r="EU15" s="11">
         <f t="shared" si="0"/>
-        <v>45895</v>
-      </c>
-      <c r="EG15" s="12">
+        <v>45986</v>
+      </c>
+      <c r="EV15" s="12">
         <f t="shared" si="0"/>
-        <v>45901</v>
-      </c>
-      <c r="EI15" s="13"/>
-      <c r="EJ15" s="17"/>
-      <c r="EK15" s="17"/>
-      <c r="EL15" s="18"/>
-      <c r="EM15" s="18"/>
-      <c r="EN15" s="17"/>
-      <c r="EO15" s="17"/>
+        <v>45992</v>
+      </c>
+      <c r="EX15" s="13"/>
+      <c r="EY15" s="17"/>
+      <c r="EZ15" s="17"/>
+      <c r="FA15" s="18"/>
+      <c r="FB15" s="18"/>
+      <c r="FC15" s="17"/>
+      <c r="FD15" s="17"/>
     </row>
-    <row r="16" spans="1:152" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:167" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="21">
         <v>12</v>
       </c>
@@ -3893,47 +4021,62 @@
       <c r="EA16" s="22"/>
       <c r="EB16" s="22"/>
       <c r="EC16" s="22"/>
-      <c r="ED16" s="26"/>
+      <c r="ED16" s="22"/>
       <c r="EE16" s="22"/>
-      <c r="EF16" s="11">
+      <c r="EF16" s="22"/>
+      <c r="EG16" s="22"/>
+      <c r="EH16" s="22"/>
+      <c r="EI16" s="22"/>
+      <c r="EJ16" s="22"/>
+      <c r="EK16" s="22"/>
+      <c r="EL16" s="22"/>
+      <c r="EM16" s="22"/>
+      <c r="EN16" s="22"/>
+      <c r="EO16" s="22"/>
+      <c r="EP16" s="22"/>
+      <c r="EQ16" s="22"/>
+      <c r="ER16" s="22"/>
+      <c r="ES16" s="26"/>
+      <c r="ET16" s="22"/>
+      <c r="EU16" s="11">
         <f t="shared" si="0"/>
-        <v>45902</v>
-      </c>
-      <c r="EG16" s="12">
+        <v>45993</v>
+      </c>
+      <c r="EV16" s="12">
         <f t="shared" si="0"/>
-        <v>45908</v>
-      </c>
-      <c r="EI16" s="13"/>
-      <c r="EJ16" s="17"/>
-      <c r="EK16" s="17"/>
-      <c r="EL16" s="18"/>
-      <c r="EM16" s="18"/>
-      <c r="EN16" s="17"/>
-      <c r="EO16" s="17"/>
+        <v>45999</v>
+      </c>
+      <c r="EX16" s="13"/>
+      <c r="EY16" s="17"/>
+      <c r="EZ16" s="17"/>
+      <c r="FA16" s="18"/>
+      <c r="FB16" s="18"/>
+      <c r="FC16" s="17"/>
+      <c r="FD16" s="17"/>
     </row>
-    <row r="17" spans="1:146" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:161" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="23"/>
-      <c r="EH17" s="13"/>
-      <c r="EI17" s="13"/>
-      <c r="EJ17" s="13"/>
-      <c r="EK17" s="17"/>
-      <c r="EL17" s="17"/>
-      <c r="EM17" s="18"/>
-      <c r="EN17" s="18"/>
-      <c r="EO17" s="17"/>
-      <c r="EP17" s="17"/>
+      <c r="EW17" s="13"/>
+      <c r="EX17" s="13"/>
+      <c r="EY17" s="13"/>
+      <c r="EZ17" s="17"/>
+      <c r="FA17" s="17"/>
+      <c r="FB17" s="18"/>
+      <c r="FC17" s="18"/>
+      <c r="FD17" s="17"/>
+      <c r="FE17" s="17"/>
     </row>
-    <row r="18" spans="1:146" x14ac:dyDescent="0.25">
-      <c r="EK18" s="17"/>
-      <c r="EL18" s="17"/>
-      <c r="EM18" s="18"/>
-      <c r="EN18" s="18"/>
-      <c r="EO18" s="17"/>
-      <c r="EP18" s="17"/>
+    <row r="18" spans="1:161" x14ac:dyDescent="0.25">
+      <c r="EZ18" s="17"/>
+      <c r="FA18" s="17"/>
+      <c r="FB18" s="18"/>
+      <c r="FC18" s="18"/>
+      <c r="FD18" s="17"/>
+      <c r="FE18" s="17"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B5:EE16">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="%">
+  <conditionalFormatting sqref="B5:ET16">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="%">
       <formula>NOT(ISERROR(SEARCH("%",B5)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>